<commit_message>
Routine image and remaining questions editing
</commit_message>
<xml_diff>
--- a/InvigilatorLlist  Of  Annual Exmination 2082 final.xlsx
+++ b/InvigilatorLlist  Of  Annual Exmination 2082 final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\Annual Exam 2082\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{425DB8C9-3A29-48E3-9C49-F2AB37AF6AF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEA20CC1-F88F-451A-8474-1B9ADBF0D5ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="64">
   <si>
     <t>GREEN SOCIETY PUBLIC SCHOOL</t>
   </si>
@@ -160,13 +160,7 @@
     <t>Nursery</t>
   </si>
   <si>
-    <t>BhawanaChapagain</t>
-  </si>
-  <si>
     <t>Apikshya Bote</t>
-  </si>
-  <si>
-    <t xml:space="preserve">        : R= Runner, C= Copy Collector</t>
   </si>
   <si>
     <t>Exam Co-ordinator</t>
@@ -266,6 +260,15 @@
   </si>
   <si>
     <t>PG</t>
+  </si>
+  <si>
+    <t>C-8</t>
+  </si>
+  <si>
+    <t>Bhawana Chapagain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        : R= Runner, C= Copy Collector, C-8 = To be facilitationg for C-8 studetns regarding BLE Exam - 2082, PG = Play Group, L = Leave</t>
   </si>
 </sst>
 </file>
@@ -323,7 +326,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -347,37 +350,9 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
+      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -387,7 +362,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -421,21 +396,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -814,46 +784,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
     </row>
     <row r="2" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
-      <c r="B2" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
+      <c r="B2" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
     </row>
     <row r="3" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
     </row>
     <row r="4" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -872,16 +842,16 @@
         <v>66822</v>
       </c>
       <c r="F4" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="I4" s="4" t="s">
         <v>46</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>48</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>4</v>
@@ -895,7 +865,9 @@
         <v>5</v>
       </c>
       <c r="C5" s="3"/>
-      <c r="D5" s="6"/>
+      <c r="D5" s="6" t="s">
+        <v>6</v>
+      </c>
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
@@ -918,10 +890,14 @@
       <c r="F6" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
+      <c r="G6" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="H6" s="6">
+        <v>7</v>
+      </c>
       <c r="I6" s="6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J6" s="6"/>
     </row>
@@ -935,13 +911,13 @@
       <c r="C7" s="2"/>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6" t="s">
+      <c r="F7" s="6" t="s">
         <v>8</v>
       </c>
+      <c r="G7" s="6"/>
       <c r="H7" s="6"/>
       <c r="I7" s="6">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J7" s="6"/>
     </row>
@@ -959,10 +935,12 @@
       <c r="E8" s="6">
         <v>4</v>
       </c>
-      <c r="F8" s="6">
-        <v>7</v>
-      </c>
-      <c r="G8" s="6"/>
+      <c r="F8" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="G8" s="6">
+        <v>4</v>
+      </c>
       <c r="H8" s="6">
         <v>6</v>
       </c>
@@ -985,8 +963,8 @@
       <c r="G9" s="6">
         <v>6</v>
       </c>
-      <c r="H9" s="6">
-        <v>7</v>
+      <c r="H9" s="6" t="s">
+        <v>61</v>
       </c>
       <c r="I9" s="6"/>
       <c r="J9" s="6"/>
@@ -1007,8 +985,8 @@
       <c r="E10" s="6">
         <v>5</v>
       </c>
-      <c r="F10" s="6" t="s">
-        <v>8</v>
+      <c r="F10" s="6">
+        <v>7</v>
       </c>
       <c r="G10" s="6">
         <v>4</v>
@@ -1052,7 +1030,7 @@
         <v>8</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C12" s="2">
         <v>1</v>
@@ -1085,8 +1063,8 @@
       <c r="C13" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D13" s="6">
-        <v>4</v>
+      <c r="D13" s="6" t="s">
+        <v>61</v>
       </c>
       <c r="E13" s="6">
         <v>7</v>
@@ -1108,7 +1086,7 @@
         <v>10</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C14" s="2">
         <v>2</v>
@@ -1136,13 +1114,13 @@
         <v>11</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C15" s="2">
         <v>6</v>
       </c>
-      <c r="D15" s="6" t="s">
-        <v>6</v>
+      <c r="D15" s="6">
+        <v>4</v>
       </c>
       <c r="E15" s="6">
         <v>2</v>
@@ -1196,7 +1174,7 @@
         <v>13</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C17" s="11">
         <v>4</v>
@@ -1208,10 +1186,10 @@
         <v>3</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H17" s="6">
         <v>5</v>
@@ -1229,16 +1207,16 @@
         <v>16</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G18" s="6" t="s">
         <v>18</v>
@@ -1257,13 +1235,13 @@
         <v>19</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>18</v>
@@ -1288,19 +1266,19 @@
         <v>22</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E20" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="G20" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F20" s="6" t="s">
+      <c r="H20" s="6" t="s">
         <v>58</v>
-      </c>
-      <c r="G20" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>60</v>
       </c>
       <c r="I20" s="6"/>
       <c r="J20" s="8"/>
@@ -1313,7 +1291,7 @@
         <v>25</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>22</v>
@@ -1344,16 +1322,16 @@
         <v>27</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>27</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="H22" s="6" t="s">
         <v>27</v>
@@ -1366,7 +1344,7 @@
         <v>19</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C23" s="11" t="s">
         <v>27</v>
@@ -1394,7 +1372,7 @@
         <v>20</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C24" s="11"/>
       <c r="D24" s="7" t="s">
@@ -1416,7 +1394,7 @@
         <v>21</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C25" s="11" t="s">
         <v>30</v>
@@ -1431,7 +1409,7 @@
         <v>27</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="H25" s="6" t="s">
         <v>30</v>
@@ -1444,7 +1422,7 @@
         <v>22</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>28</v>
@@ -1528,7 +1506,7 @@
         <v>25</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>32</v>
@@ -1556,7 +1534,7 @@
         <v>26</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>32</v>
@@ -1584,7 +1562,7 @@
         <v>27</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>32</v>
@@ -1612,7 +1590,7 @@
         <v>28</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>32</v>
@@ -1640,34 +1618,34 @@
         <v>29</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H33" s="11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I33" s="11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J33" s="8"/>
     </row>
     <row r="34" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="13" t="s">
-        <v>41</v>
+      <c r="A34" s="14" t="s">
+        <v>39</v>
       </c>
       <c r="B34" s="14"/>
       <c r="C34" s="14"/>
@@ -1677,33 +1655,36 @@
       <c r="G34" s="14"/>
       <c r="H34" s="14"/>
       <c r="I34" s="14"/>
-      <c r="J34" s="15"/>
+      <c r="J34" s="14"/>
     </row>
     <row r="35" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="B35" s="17"/>
-      <c r="C35" s="17"/>
-      <c r="D35" s="17"/>
-      <c r="E35" s="17"/>
-      <c r="F35" s="17"/>
-      <c r="G35" s="17"/>
-      <c r="H35" s="17"/>
-      <c r="I35" s="17"/>
-      <c r="J35" s="17"/>
+      <c r="A35" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="B35" s="15"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
+      <c r="H35" s="15"/>
+      <c r="I35" s="15"/>
+      <c r="J35" s="15"/>
     </row>
     <row r="36" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I36" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="J36" s="12"/>
-    </row>
-    <row r="37" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="I36" s="16"/>
+      <c r="J36" s="16"/>
+    </row>
+    <row r="37" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I37" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="J37" s="12"/>
+    </row>
     <row r="38" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="I36:J36"/>
+    <mergeCell ref="I37:J37"/>
     <mergeCell ref="A34:J34"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="B2:J2"/>

</xml_diff>

<commit_message>
D-15 sent for printing
</commit_message>
<xml_diff>
--- a/InvigilatorLlist  Of  Annual Exmination 2082 final.xlsx
+++ b/InvigilatorLlist  Of  Annual Exmination 2082 final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\Annual Exam 2082\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEA20CC1-F88F-451A-8474-1B9ADBF0D5ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57358C56-F688-469D-8747-6B8078A270F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="64">
   <si>
     <t>GREEN SOCIETY PUBLIC SCHOOL</t>
   </si>
@@ -393,19 +393,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -784,46 +784,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
     </row>
     <row r="4" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -908,13 +908,17 @@
       <c r="B7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="2"/>
+      <c r="C7" s="7" t="s">
+        <v>61</v>
+      </c>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
       <c r="F7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G7" s="6"/>
+      <c r="G7" s="7" t="s">
+        <v>61</v>
+      </c>
       <c r="H7" s="6"/>
       <c r="I7" s="6">
         <v>7</v>
@@ -959,9 +963,11 @@
       <c r="C9" s="2"/>
       <c r="D9" s="6"/>
       <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
+      <c r="F9" s="6">
+        <v>6</v>
+      </c>
       <c r="G9" s="6">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>61</v>
@@ -1045,7 +1051,7 @@
         <v>4</v>
       </c>
       <c r="G12" s="6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H12" s="6"/>
       <c r="I12" s="6">
@@ -1070,12 +1076,14 @@
         <v>7</v>
       </c>
       <c r="F13" s="6">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G13" s="6">
         <v>2</v>
       </c>
-      <c r="H13" s="6"/>
+      <c r="H13" s="6">
+        <v>2</v>
+      </c>
       <c r="I13" s="6">
         <v>3</v>
       </c>
@@ -1125,9 +1133,7 @@
       <c r="E15" s="6">
         <v>2</v>
       </c>
-      <c r="F15" s="6">
-        <v>3</v>
-      </c>
+      <c r="F15" s="6"/>
       <c r="G15" s="6">
         <v>5</v>
       </c>
@@ -1161,9 +1167,7 @@
       <c r="G16" s="6">
         <v>1</v>
       </c>
-      <c r="H16" s="6">
-        <v>2</v>
-      </c>
+      <c r="H16" s="6"/>
       <c r="I16" s="6">
         <v>4</v>
       </c>
@@ -1658,28 +1662,28 @@
       <c r="J34" s="14"/>
     </row>
     <row r="35" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="15" t="s">
+      <c r="A35" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="B35" s="15"/>
-      <c r="C35" s="15"/>
-      <c r="D35" s="15"/>
-      <c r="E35" s="15"/>
-      <c r="F35" s="15"/>
-      <c r="G35" s="15"/>
-      <c r="H35" s="15"/>
-      <c r="I35" s="15"/>
-      <c r="J35" s="15"/>
+      <c r="B35" s="16"/>
+      <c r="C35" s="16"/>
+      <c r="D35" s="16"/>
+      <c r="E35" s="16"/>
+      <c r="F35" s="16"/>
+      <c r="G35" s="16"/>
+      <c r="H35" s="16"/>
+      <c r="I35" s="16"/>
+      <c r="J35" s="16"/>
     </row>
     <row r="36" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I36" s="16"/>
-      <c r="J36" s="16"/>
+      <c r="I36" s="12"/>
+      <c r="J36" s="12"/>
     </row>
     <row r="37" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I37" s="12" t="s">
+      <c r="I37" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="J37" s="12"/>
+      <c r="J37" s="13"/>
     </row>
     <row r="38" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>

</xml_diff>